<commit_message>
File re-org and cleanup
</commit_message>
<xml_diff>
--- a/admin/SciComp-Demos - Parts List - Sensors.xlsx
+++ b/admin/SciComp-Demos - Parts List - Sensors.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DaveB\Repos\scicomp-demos\admin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DaveB\SciComp\Courses\scicomp-demos\_archive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388DCD20-1559-4BEF-A4AF-023519E484E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027AFAB6-06F5-457A-A9F1-FE57F9BCB9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{33F6F95C-2D53-4E62-A210-0FCD4640A9B8}"/>
   </bookViews>
@@ -278,7 +278,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -309,6 +309,12 @@
     <xf numFmtId="8" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -735,8 +741,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1B15000B-C80C-4FAD-949F-AB73D2A1A9B8}" name="Table4" displayName="Table4" ref="B63:H72" totalsRowCount="1" headerRowDxfId="10">
-  <autoFilter ref="B63:H71" xr:uid="{1B15000B-C80C-4FAD-949F-AB73D2A1A9B8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1B15000B-C80C-4FAD-949F-AB73D2A1A9B8}" name="Table4" displayName="Table4" ref="B64:H73" totalsRowCount="1" headerRowDxfId="10">
+  <autoFilter ref="B64:H72" xr:uid="{1B15000B-C80C-4FAD-949F-AB73D2A1A9B8}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{DAFCF0FF-D9BF-4CEF-834B-3406E64AD0D1}" name="Element ID" dataDxfId="9" totalsRowDxfId="8"/>
     <tableColumn id="2" xr3:uid="{73C9EAF7-C709-4AD0-AFC7-0D169ABA564F}" name="Design ID" dataDxfId="7" totalsRowDxfId="6"/>
@@ -745,7 +751,7 @@
     <tableColumn id="5" xr3:uid="{6C4FC6E9-D7B0-451F-AB3D-2BEE180A3DB1}" name="Qty" dataDxfId="5" totalsRowDxfId="4"/>
     <tableColumn id="6" xr3:uid="{7ED7C766-980B-4488-98FB-2D4156B57C18}" name="Unit Cost" dataDxfId="3" totalsRowDxfId="2" dataCellStyle="Currency" totalsRowCellStyle="Currency"/>
     <tableColumn id="7" xr3:uid="{7D4587FC-F9C3-4F92-B73A-59C29101E5F1}" name="Total Cost" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0" dataCellStyle="Currency" totalsRowCellStyle="Currency">
-      <calculatedColumnFormula>+F64*G64</calculatedColumnFormula>
+      <calculatedColumnFormula>+F65*G65</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1049,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7AB3C2-C500-46AF-BB74-509C61346243}">
-  <dimension ref="B2:H75"/>
+  <dimension ref="B2:H76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="18.42578125" customWidth="1"/>
@@ -2026,274 +2032,278 @@
       </c>
     </row>
     <row r="58" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C58" s="2" t="s">
+      <c r="C58" s="16" t="s">
         <v>43</v>
       </c>
+      <c r="D58" s="16"/>
       <c r="E58" s="13">
         <v>64.95</v>
       </c>
     </row>
     <row r="59" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C59" s="2" t="s">
+      <c r="C59" s="16" t="s">
         <v>44</v>
       </c>
+      <c r="D59" s="16"/>
       <c r="E59" s="13">
         <v>1.95</v>
       </c>
     </row>
     <row r="60" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="17" t="s">
         <v>45</v>
       </c>
+      <c r="D60" s="17"/>
       <c r="E60" s="13">
         <v>32.1</v>
       </c>
     </row>
     <row r="61" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="17" t="s">
         <v>46</v>
       </c>
+      <c r="D61" s="17"/>
       <c r="E61" s="13">
         <v>7.12</v>
       </c>
     </row>
     <row r="62" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="17" t="s">
         <v>47</v>
       </c>
+      <c r="D62" s="17"/>
       <c r="E62" s="13">
         <v>28.95</v>
       </c>
     </row>
     <row r="63" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
+      <c r="C63" s="6"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="13"/>
+    </row>
+    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
         <v>11</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C64" t="s">
         <v>12</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D64" t="s">
         <v>1</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E64" t="s">
         <v>5</v>
       </c>
-      <c r="F63" s="7" t="s">
+      <c r="F64" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G63" s="7" t="s">
+      <c r="G64" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H63" s="7" t="s">
+      <c r="H64" s="7" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B64" s="1">
-        <v>300326</v>
-      </c>
-      <c r="C64" s="1">
-        <v>3003</v>
-      </c>
-      <c r="D64" t="s">
-        <v>48</v>
-      </c>
-      <c r="E64" t="s">
-        <v>6</v>
-      </c>
-      <c r="F64" s="7">
-        <v>10</v>
-      </c>
-      <c r="G64" s="10">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="H64" s="3">
-        <f>+F64*G64</f>
-        <v>1.4000000000000001</v>
       </c>
     </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B65" s="1">
-        <v>300226</v>
+        <v>300326</v>
       </c>
       <c r="C65" s="1">
-        <v>3002</v>
+        <v>3003</v>
       </c>
       <c r="D65" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E65" t="s">
         <v>6</v>
       </c>
       <c r="F65" s="7">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G65" s="10">
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="H65" s="3">
-        <f t="shared" ref="H65:H71" si="1">+F65*G65</f>
-        <v>0.34</v>
+        <f>+F65*G65</f>
+        <v>1.4000000000000001</v>
       </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B66" s="1">
-        <v>300926</v>
+        <v>300226</v>
       </c>
       <c r="C66" s="1">
-        <v>3009</v>
+        <v>3002</v>
       </c>
       <c r="D66" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E66" t="s">
         <v>6</v>
       </c>
       <c r="F66" s="7">
+        <v>2</v>
+      </c>
+      <c r="G66" s="10">
+        <v>0.17</v>
+      </c>
+      <c r="H66" s="3">
+        <f t="shared" ref="H66:H72" si="1">+F66*G66</f>
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B67" s="1">
+        <v>300926</v>
+      </c>
+      <c r="C67" s="1">
+        <v>3009</v>
+      </c>
+      <c r="D67" t="s">
+        <v>50</v>
+      </c>
+      <c r="E67" t="s">
+        <v>6</v>
+      </c>
+      <c r="F67" s="7">
         <v>3</v>
       </c>
-      <c r="G66" s="10">
+      <c r="G67" s="10">
         <v>0.25</v>
       </c>
-      <c r="H66" s="3">
+      <c r="H67" s="3">
         <f t="shared" si="1"/>
         <v>0.75</v>
       </c>
     </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B67" s="1">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B68" s="1">
         <v>300426</v>
       </c>
-      <c r="C67" s="1">
+      <c r="C68" s="1">
         <v>3004</v>
       </c>
-      <c r="D67" t="s">
+      <c r="D68" t="s">
         <v>18</v>
       </c>
-      <c r="E67" t="s">
+      <c r="E68" t="s">
         <v>6</v>
       </c>
-      <c r="F67" s="7">
+      <c r="F68" s="7">
         <v>2</v>
       </c>
-      <c r="G67" s="10">
+      <c r="G68" s="10">
         <v>0.11</v>
       </c>
-      <c r="H67" s="3">
+      <c r="H68" s="3">
         <f t="shared" si="1"/>
         <v>0.22</v>
       </c>
     </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B68" s="1">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B69" s="1">
         <v>303226</v>
       </c>
-      <c r="C68" s="1">
+      <c r="C69" s="1">
         <v>3032</v>
       </c>
-      <c r="D68" t="s">
+      <c r="D69" t="s">
         <v>26</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E69" t="s">
         <v>6</v>
       </c>
-      <c r="F68" s="7">
+      <c r="F69" s="7">
         <v>1</v>
       </c>
-      <c r="G68" s="10">
+      <c r="G69" s="10">
         <v>0.43</v>
       </c>
-      <c r="H68" s="3">
+      <c r="H69" s="3">
         <f t="shared" si="1"/>
         <v>0.43</v>
       </c>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B69" s="1">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B70" s="1">
         <v>303426</v>
       </c>
-      <c r="C69" s="1">
+      <c r="C70" s="1">
         <v>3034</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D70" t="s">
         <v>35</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E70" t="s">
         <v>6</v>
       </c>
-      <c r="F69" s="7">
+      <c r="F70" s="7">
         <v>1</v>
       </c>
-      <c r="G69" s="10">
+      <c r="G70" s="10">
         <v>0.25</v>
       </c>
-      <c r="H69" s="3">
+      <c r="H70" s="3">
         <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
     </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B70" s="1">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B71" s="1">
         <v>303526</v>
       </c>
-      <c r="C70" s="1">
+      <c r="C71" s="1">
         <v>3035</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D71" t="s">
         <v>51</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E71" t="s">
         <v>6</v>
       </c>
-      <c r="F70" s="7">
+      <c r="F71" s="7">
         <v>1</v>
       </c>
-      <c r="G70" s="10">
+      <c r="G71" s="10">
         <v>0.46</v>
       </c>
-      <c r="H70" s="3">
+      <c r="H71" s="3">
         <f t="shared" si="1"/>
         <v>0.46</v>
       </c>
     </row>
-    <row r="71" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B71" s="1">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B72" s="1">
         <v>243121</v>
       </c>
-      <c r="C71" s="1">
+      <c r="C72" s="1">
         <v>2431</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D72" t="s">
         <v>52</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E72" t="s">
         <v>17</v>
       </c>
-      <c r="F71" s="7">
+      <c r="F72" s="7">
         <v>2</v>
       </c>
-      <c r="G71" s="10">
+      <c r="G72" s="10">
         <v>0.13</v>
       </c>
-      <c r="H71" s="3">
+      <c r="H72" s="3">
         <f t="shared" si="1"/>
         <v>0.26</v>
-      </c>
-    </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-      <c r="G72" s="10"/>
-      <c r="H72" s="15">
-        <f>SUBTOTAL(109,Table4[Total Cost])</f>
-        <v>4.1100000000000003</v>
       </c>
     </row>
     <row r="73" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
       <c r="G73" s="10"/>
-      <c r="H73" s="3"/>
+      <c r="H73" s="15">
+        <f>SUBTOTAL(109,Table4[Total Cost])</f>
+        <v>4.1100000000000003</v>
+      </c>
     </row>
     <row r="74" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
@@ -2307,7 +2317,20 @@
       <c r="G75" s="10"/>
       <c r="H75" s="3"/>
     </row>
+    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+      <c r="G76" s="10"/>
+      <c r="H76" s="3"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C62:D62"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{17EF0979-152B-4972-9745-8AAEE713699A}"/>
     <hyperlink ref="C9" r:id="rId2" xr:uid="{8ED3F0F8-EBFB-43AC-8BD0-C2BAE22CF7E4}"/>

</xml_diff>